<commit_message>
feat: add new mission creation page and update schema
- Introduced a new page for creating missions with a multi-step form.
- Updated Prisma schema to include new fields and relations for the Mission model.
- Added validation schemas for mission creation steps.
- Enhanced UI components for better user experience in the dashboard.
- Updated various pages to use consistent typography components.
- Added a new PDF document for Renford incoherences.
</commit_message>
<xml_diff>
--- a/Docs/Cartographie _ Type de mission _ Renford.xlsx
+++ b/Docs/Cartographie _ Type de mission _ Renford.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cc5693273bc23704/Documents/Renford/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Desktop\Dev Projects\renford\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{353F3CAB-E94A-4BA3-9FE6-AD552E05A914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3797E483-2768-4395-82C5-41567BF87B6F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AAB268C-EE10-4194-AF22-07BF3F114FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catégorie" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="Spécialité" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="120">
   <si>
     <t>ID_Catégorie</t>
   </si>
@@ -378,13 +377,31 @@
   </si>
   <si>
     <t>Hot Yoga</t>
+  </si>
+  <si>
+    <t>Boxe &amp; Arts martiaux</t>
+  </si>
+  <si>
+    <t>Zumba</t>
+  </si>
+  <si>
+    <t>Programmes les mills</t>
+  </si>
+  <si>
+    <t>Animation sportive &amp; Multisport</t>
+  </si>
+  <si>
+    <t>Bien-être &amp; Sport santé</t>
+  </si>
+  <si>
+    <t>Discipline</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -409,6 +426,21 @@
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -430,7 +462,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -438,6 +470,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="10"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,10 +487,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -661,12 +691,12 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="32.7265625" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -674,7 +704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -682,7 +712,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -690,7 +720,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -698,7 +728,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -706,7 +736,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -714,7 +744,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -722,7 +752,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -730,7 +760,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -746,14 +776,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32E4EEF3-2D0D-417C-98C3-18C6B9A0DDAB}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>81</v>
       </c>
@@ -767,7 +797,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>3</v>
       </c>
@@ -781,7 +811,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
       <c r="C3" t="s">
@@ -791,39 +821,39 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
     </row>
-    <row r="7" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="2"/>
     </row>
@@ -838,14 +868,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:D93"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="42.90625" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" customWidth="1"/>
-    <col min="4" max="4" width="21.36328125" customWidth="1"/>
+    <col min="2" max="2" width="42.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -855,8 +885,11 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D1" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -866,8 +899,11 @@
       <c r="C2" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -877,23 +913,11 @@
       <c r="C3" s="2">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="str">
-        <f t="shared" ref="D3:D34" si="0">IF(C3="Pilates",1,
-IF(C3="Yoga",2,
-IF(C3="Fitness &amp; Musculation",3,
-IF(C3="Escalade",5,
-IF(C3="Boxe",6,
-IF(C3="Danse",7,
-IF(C3="Gymnastique",8,
-IF(C3="Activité Physique Adaptée (APA)",9,
-IF(C3="Bien-Être &amp; Récupération",10,
-IF(C3="Activités aquatiques",11,
-IF(C3="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -903,9 +927,11 @@
       <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -915,12 +941,11 @@
       <c r="C5" s="2">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -930,12 +955,11 @@
       <c r="C6" s="2">
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -945,12 +969,11 @@
       <c r="C7" s="2">
         <v>1</v>
       </c>
-      <c r="D7" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -960,12 +983,11 @@
       <c r="C8" s="2">
         <v>1</v>
       </c>
-      <c r="D8" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -975,12 +997,11 @@
       <c r="C9" s="2">
         <v>1</v>
       </c>
-      <c r="D9" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -990,12 +1011,11 @@
       <c r="C10" s="2">
         <v>2</v>
       </c>
-      <c r="D10" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D10" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1005,12 +1025,11 @@
       <c r="C11" s="2">
         <v>2</v>
       </c>
-      <c r="D11" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D11" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1020,12 +1039,11 @@
       <c r="C12" s="2">
         <v>2</v>
       </c>
-      <c r="D12" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1035,12 +1053,11 @@
       <c r="C13" s="2">
         <v>2</v>
       </c>
-      <c r="D13" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D13" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1050,9 +1067,11 @@
       <c r="C14" s="2">
         <v>2</v>
       </c>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1062,12 +1081,11 @@
       <c r="C15" s="2">
         <v>2</v>
       </c>
-      <c r="D15" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D15" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1077,12 +1095,11 @@
       <c r="C16" s="2">
         <v>2</v>
       </c>
-      <c r="D16" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D16" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1092,12 +1109,11 @@
       <c r="C17" s="2">
         <v>2</v>
       </c>
-      <c r="D17" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D17" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1107,12 +1123,11 @@
       <c r="C18" s="2">
         <v>2</v>
       </c>
-      <c r="D18" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D18" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1122,12 +1137,11 @@
       <c r="C19" s="2">
         <v>2</v>
       </c>
-      <c r="D19" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D19" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1137,12 +1151,11 @@
       <c r="C20" s="2">
         <v>3</v>
       </c>
-      <c r="D20" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D20" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1152,12 +1165,11 @@
       <c r="C21" s="2">
         <v>3</v>
       </c>
-      <c r="D21" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D21" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1167,12 +1179,11 @@
       <c r="C22" s="2">
         <v>3</v>
       </c>
-      <c r="D22" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1182,12 +1193,11 @@
       <c r="C23" s="2">
         <v>3</v>
       </c>
-      <c r="D23" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D23" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1197,12 +1207,11 @@
       <c r="C24" s="2">
         <v>3</v>
       </c>
-      <c r="D24" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D24" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1212,12 +1221,11 @@
       <c r="C25" s="2">
         <v>3</v>
       </c>
-      <c r="D25" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D25" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1227,12 +1235,11 @@
       <c r="C26" s="2">
         <v>3</v>
       </c>
-      <c r="D26" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D26" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1242,12 +1249,11 @@
       <c r="C27" s="2">
         <v>3</v>
       </c>
-      <c r="D27" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D27" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -1257,12 +1263,11 @@
       <c r="C28" s="2">
         <v>3</v>
       </c>
-      <c r="D28" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D28" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1272,12 +1277,11 @@
       <c r="C29" s="2">
         <v>3</v>
       </c>
-      <c r="D29" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D29" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -1287,12 +1291,11 @@
       <c r="C30" s="2">
         <v>3</v>
       </c>
-      <c r="D30" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D30" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1302,12 +1305,11 @@
       <c r="C31" s="2">
         <v>3</v>
       </c>
-      <c r="D31" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D31" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -1317,12 +1319,11 @@
       <c r="C32" s="2">
         <v>3</v>
       </c>
-      <c r="D32" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D32" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -1332,12 +1333,11 @@
       <c r="C33" s="2">
         <v>3</v>
       </c>
-      <c r="D33" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D33" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -1347,12 +1347,11 @@
       <c r="C34" s="2">
         <v>3</v>
       </c>
-      <c r="D34" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D34" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -1362,9 +1361,11 @@
       <c r="C35" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D35" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -1374,9 +1375,11 @@
       <c r="C36" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D36" s="2"/>
-    </row>
-    <row r="37" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D36" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -1386,9 +1389,11 @@
       <c r="C37" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D37" s="2"/>
-    </row>
-    <row r="38" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D37" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -1398,9 +1403,11 @@
       <c r="C38" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D38" s="2"/>
-    </row>
-    <row r="39" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D38" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -1410,9 +1417,11 @@
       <c r="C39" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D39" s="2"/>
-    </row>
-    <row r="40" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D39" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -1422,9 +1431,11 @@
       <c r="C40" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D40" s="2"/>
-    </row>
-    <row r="41" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D40" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -1434,9 +1445,11 @@
       <c r="C41" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D41" s="2"/>
-    </row>
-    <row r="42" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D41" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -1446,9 +1459,11 @@
       <c r="C42" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D42" s="2"/>
-    </row>
-    <row r="43" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D42" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -1458,23 +1473,11 @@
       <c r="C43" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D43" s="2" t="str">
-        <f>IF(C57="Pilates",1,
-IF(C57="Yoga",2,
-IF(C57="Fitness &amp; Musculation",3,
-IF(C57="Escalade",5,
-IF(C57="Boxe",6,
-IF(C57="Danse",7,
-IF(C57="Gymnastique",8,
-IF(C57="Activité Physique Adaptée (APA)",9,
-IF(C57="Bien-Être &amp; Récupération",10,
-IF(C57="Activités aquatiques",11,
-IF(C57="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D43" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -1484,23 +1487,11 @@
       <c r="C44" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D44" s="2" t="str">
-        <f>IF(C58="Pilates",1,
-IF(C58="Yoga",2,
-IF(C58="Fitness &amp; Musculation",3,
-IF(C58="Escalade",5,
-IF(C58="Boxe",6,
-IF(C58="Danse",7,
-IF(C58="Gymnastique",8,
-IF(C58="Activité Physique Adaptée (APA)",9,
-IF(C58="Bien-Être &amp; Récupération",10,
-IF(C58="Activités aquatiques",11,
-IF(C58="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D44" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -1510,23 +1501,11 @@
       <c r="C45" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D45" s="2" t="str">
-        <f>IF(C59="Pilates",1,
-IF(C59="Yoga",2,
-IF(C59="Fitness &amp; Musculation",3,
-IF(C59="Escalade",5,
-IF(C59="Boxe",6,
-IF(C59="Danse",7,
-IF(C59="Gymnastique",8,
-IF(C59="Activité Physique Adaptée (APA)",9,
-IF(C59="Bien-Être &amp; Récupération",10,
-IF(C59="Activités aquatiques",11,
-IF(C59="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D45" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -1536,23 +1515,11 @@
       <c r="C46" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D46" s="2" t="str">
-        <f>IF(C60="Pilates",1,
-IF(C60="Yoga",2,
-IF(C60="Fitness &amp; Musculation",3,
-IF(C60="Escalade",5,
-IF(C60="Boxe",6,
-IF(C60="Danse",7,
-IF(C60="Gymnastique",8,
-IF(C60="Activité Physique Adaptée (APA)",9,
-IF(C60="Bien-Être &amp; Récupération",10,
-IF(C60="Activités aquatiques",11,
-IF(C60="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D46" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -1562,23 +1529,11 @@
       <c r="C47" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D47" s="2" t="str">
-        <f>IF(C61="Pilates",1,
-IF(C61="Yoga",2,
-IF(C61="Fitness &amp; Musculation",3,
-IF(C61="Escalade",5,
-IF(C61="Boxe",6,
-IF(C61="Danse",7,
-IF(C61="Gymnastique",8,
-IF(C61="Activité Physique Adaptée (APA)",9,
-IF(C61="Bien-Être &amp; Récupération",10,
-IF(C61="Activités aquatiques",11,
-IF(C61="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D47" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -1588,9 +1543,11 @@
       <c r="C48" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D48" s="2"/>
-    </row>
-    <row r="49" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D48" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -1600,23 +1557,11 @@
       <c r="C49" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D49" s="2" t="str">
-        <f>IF(C62="Pilates",1,
-IF(C62="Yoga",2,
-IF(C62="Fitness &amp; Musculation",3,
-IF(C62="Escalade",5,
-IF(C62="Boxe",6,
-IF(C62="Danse",7,
-IF(C62="Gymnastique",8,
-IF(C62="Activité Physique Adaptée (APA)",9,
-IF(C62="Bien-Être &amp; Récupération",10,
-IF(C62="Activités aquatiques",11,
-IF(C62="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D49" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -1626,23 +1571,11 @@
       <c r="C50" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D50" s="2" t="str">
-        <f>IF(C63="Pilates",1,
-IF(C63="Yoga",2,
-IF(C63="Fitness &amp; Musculation",3,
-IF(C63="Escalade",5,
-IF(C63="Boxe",6,
-IF(C63="Danse",7,
-IF(C63="Gymnastique",8,
-IF(C63="Activité Physique Adaptée (APA)",9,
-IF(C63="Bien-Être &amp; Récupération",10,
-IF(C63="Activités aquatiques",11,
-IF(C63="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D50" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>50</v>
       </c>
@@ -1652,23 +1585,11 @@
       <c r="C51" s="2">
         <v>4</v>
       </c>
-      <c r="D51" s="2" t="str">
-        <f>IF(C65="Pilates",1,
-IF(C65="Yoga",2,
-IF(C65="Fitness &amp; Musculation",3,
-IF(C65="Escalade",5,
-IF(C65="Boxe",6,
-IF(C65="Danse",7,
-IF(C65="Gymnastique",8,
-IF(C65="Activité Physique Adaptée (APA)",9,
-IF(C65="Bien-Être &amp; Récupération",10,
-IF(C65="Activités aquatiques",11,
-IF(C65="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D51" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>51</v>
       </c>
@@ -1678,23 +1599,11 @@
       <c r="C52" s="2">
         <v>4</v>
       </c>
-      <c r="D52" s="2" t="str">
-        <f>IF(C69="Pilates",1,
-IF(C69="Yoga",2,
-IF(C69="Fitness &amp; Musculation",3,
-IF(C69="Escalade",5,
-IF(C69="Boxe",6,
-IF(C69="Danse",7,
-IF(C69="Gymnastique",8,
-IF(C69="Activité Physique Adaptée (APA)",9,
-IF(C69="Bien-Être &amp; Récupération",10,
-IF(C69="Activités aquatiques",11,
-IF(C69="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D52" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -1704,23 +1613,11 @@
       <c r="C53" s="2">
         <v>4</v>
       </c>
-      <c r="D53" s="2" t="str">
-        <f>IF(C70="Pilates",1,
-IF(C70="Yoga",2,
-IF(C70="Fitness &amp; Musculation",3,
-IF(C70="Escalade",5,
-IF(C70="Boxe",6,
-IF(C70="Danse",7,
-IF(C70="Gymnastique",8,
-IF(C70="Activité Physique Adaptée (APA)",9,
-IF(C70="Bien-Être &amp; Récupération",10,
-IF(C70="Activités aquatiques",11,
-IF(C70="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D53" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -1730,23 +1627,11 @@
       <c r="C54" s="2">
         <v>4</v>
       </c>
-      <c r="D54" s="2" t="str">
-        <f>IF(C71="Pilates",1,
-IF(C71="Yoga",2,
-IF(C71="Fitness &amp; Musculation",3,
-IF(C71="Escalade",5,
-IF(C71="Boxe",6,
-IF(C71="Danse",7,
-IF(C71="Gymnastique",8,
-IF(C71="Activité Physique Adaptée (APA)",9,
-IF(C71="Bien-Être &amp; Récupération",10,
-IF(C71="Activités aquatiques",11,
-IF(C71="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D54" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -1756,23 +1641,11 @@
       <c r="C55" s="2">
         <v>4</v>
       </c>
-      <c r="D55" s="2" t="str">
-        <f>IF(C72="Pilates",1,
-IF(C72="Yoga",2,
-IF(C72="Fitness &amp; Musculation",3,
-IF(C72="Escalade",5,
-IF(C72="Boxe",6,
-IF(C72="Danse",7,
-IF(C72="Gymnastique",8,
-IF(C72="Activité Physique Adaptée (APA)",9,
-IF(C72="Bien-Être &amp; Récupération",10,
-IF(C72="Activités aquatiques",11,
-IF(C72="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D55" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -1782,23 +1655,11 @@
       <c r="C56" s="2">
         <v>4</v>
       </c>
-      <c r="D56" s="2" t="str">
-        <f>IF(C74="Pilates",1,
-IF(C74="Yoga",2,
-IF(C74="Fitness &amp; Musculation",3,
-IF(C74="Escalade",5,
-IF(C74="Boxe",6,
-IF(C74="Danse",7,
-IF(C74="Gymnastique",8,
-IF(C74="Activité Physique Adaptée (APA)",9,
-IF(C74="Bien-Être &amp; Récupération",10,
-IF(C74="Activités aquatiques",11,
-IF(C74="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D56" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -1808,23 +1669,11 @@
       <c r="C57" s="2">
         <v>5</v>
       </c>
-      <c r="D57" s="2" t="str">
-        <f>IF(C75="Pilates",1,
-IF(C75="Yoga",2,
-IF(C75="Fitness &amp; Musculation",3,
-IF(C75="Escalade",5,
-IF(C75="Boxe",6,
-IF(C75="Danse",7,
-IF(C75="Gymnastique",8,
-IF(C75="Activité Physique Adaptée (APA)",9,
-IF(C75="Bien-Être &amp; Récupération",10,
-IF(C75="Activités aquatiques",11,
-IF(C75="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D57" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -1834,23 +1683,11 @@
       <c r="C58" s="2">
         <v>5</v>
       </c>
-      <c r="D58" s="2" t="str">
-        <f>IF(C76="Pilates",1,
-IF(C76="Yoga",2,
-IF(C76="Fitness &amp; Musculation",3,
-IF(C76="Escalade",5,
-IF(C76="Boxe",6,
-IF(C76="Danse",7,
-IF(C76="Gymnastique",8,
-IF(C76="Activité Physique Adaptée (APA)",9,
-IF(C76="Bien-Être &amp; Récupération",10,
-IF(C76="Activités aquatiques",11,
-IF(C76="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D58" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -1860,23 +1697,11 @@
       <c r="C59" s="2">
         <v>5</v>
       </c>
-      <c r="D59" s="2" t="str">
-        <f>IF(C77="Pilates",1,
-IF(C77="Yoga",2,
-IF(C77="Fitness &amp; Musculation",3,
-IF(C77="Escalade",5,
-IF(C77="Boxe",6,
-IF(C77="Danse",7,
-IF(C77="Gymnastique",8,
-IF(C77="Activité Physique Adaptée (APA)",9,
-IF(C77="Bien-Être &amp; Récupération",10,
-IF(C77="Activités aquatiques",11,
-IF(C77="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D59" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -1886,9 +1711,11 @@
       <c r="C60" s="2">
         <v>5</v>
       </c>
-      <c r="D60" s="2"/>
-    </row>
-    <row r="61" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D60" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -1898,9 +1725,11 @@
       <c r="C61" s="2">
         <v>5</v>
       </c>
-      <c r="D61" s="2"/>
-    </row>
-    <row r="62" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D61" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>61</v>
       </c>
@@ -1910,9 +1739,11 @@
       <c r="C62" s="2">
         <v>5</v>
       </c>
-      <c r="D62" s="2"/>
-    </row>
-    <row r="63" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D62" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>62</v>
       </c>
@@ -1922,23 +1753,11 @@
       <c r="C63" s="2">
         <v>6</v>
       </c>
-      <c r="D63" s="2" t="str">
-        <f>IF(C78="Pilates",1,
-IF(C78="Yoga",2,
-IF(C78="Fitness &amp; Musculation",3,
-IF(C78="Escalade",5,
-IF(C78="Boxe",6,
-IF(C78="Danse",7,
-IF(C78="Gymnastique",8,
-IF(C78="Activité Physique Adaptée (APA)",9,
-IF(C78="Bien-Être &amp; Récupération",10,
-IF(C78="Activités aquatiques",11,
-IF(C78="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D63" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>63</v>
       </c>
@@ -1948,23 +1767,11 @@
       <c r="C64" s="2">
         <v>6</v>
       </c>
-      <c r="D64" s="2" t="str">
-        <f>IF(C42="Pilates",1,
-IF(C42="Yoga",2,
-IF(C42="Fitness &amp; Musculation",3,
-IF(C42="Escalade",5,
-IF(C42="Boxe",6,
-IF(C42="Danse",7,
-IF(C42="Gymnastique",8,
-IF(C42="Activité Physique Adaptée (APA)",9,
-IF(C42="Bien-Être &amp; Récupération",10,
-IF(C42="Activités aquatiques",11,
-IF(C42="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D64" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>64</v>
       </c>
@@ -1974,8 +1781,11 @@
       <c r="C65" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D65" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>65</v>
       </c>
@@ -1985,8 +1795,11 @@
       <c r="C66" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D66" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>66</v>
       </c>
@@ -1996,8 +1809,11 @@
       <c r="C67" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D67" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>67</v>
       </c>
@@ -2007,8 +1823,11 @@
       <c r="C68" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D68" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -2018,8 +1837,11 @@
       <c r="C69" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D69" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>69</v>
       </c>
@@ -2029,8 +1851,11 @@
       <c r="C70" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D70" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>70</v>
       </c>
@@ -2040,8 +1865,11 @@
       <c r="C71" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D71" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>71</v>
       </c>
@@ -2051,8 +1879,11 @@
       <c r="C72" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D72" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>72</v>
       </c>
@@ -2062,23 +1893,11 @@
       <c r="C73" s="2">
         <v>7</v>
       </c>
-      <c r="D73" s="2" t="str">
-        <f t="shared" ref="D73:D87" si="1">IF(C79="Pilates",1,
-IF(C79="Yoga",2,
-IF(C79="Fitness &amp; Musculation",3,
-IF(C79="Escalade",5,
-IF(C79="Boxe",6,
-IF(C79="Danse",7,
-IF(C79="Gymnastique",8,
-IF(C79="Activité Physique Adaptée (APA)",9,
-IF(C79="Bien-Être &amp; Récupération",10,
-IF(C79="Activités aquatiques",11,
-IF(C79="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D73" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>73</v>
       </c>
@@ -2088,12 +1907,11 @@
       <c r="C74" s="2">
         <v>7</v>
       </c>
-      <c r="D74" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D74" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>74</v>
       </c>
@@ -2103,12 +1921,11 @@
       <c r="C75" s="2">
         <v>7</v>
       </c>
-      <c r="D75" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D75" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>75</v>
       </c>
@@ -2118,12 +1935,11 @@
       <c r="C76" s="2">
         <v>7</v>
       </c>
-      <c r="D76" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D76" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>76</v>
       </c>
@@ -2133,12 +1949,11 @@
       <c r="C77" s="2">
         <v>7</v>
       </c>
-      <c r="D77" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D77" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>77</v>
       </c>
@@ -2148,12 +1963,11 @@
       <c r="C78" s="2">
         <v>7</v>
       </c>
-      <c r="D78" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D78" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>78</v>
       </c>
@@ -2163,12 +1977,11 @@
       <c r="C79" s="2">
         <v>7</v>
       </c>
-      <c r="D79" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D79" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>79</v>
       </c>
@@ -2178,12 +1991,11 @@
       <c r="C80" s="2">
         <v>7</v>
       </c>
-      <c r="D80" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D80" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>80</v>
       </c>
@@ -2193,12 +2005,11 @@
       <c r="C81" s="2">
         <v>7</v>
       </c>
-      <c r="D81" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D81" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>81</v>
       </c>
@@ -2208,12 +2019,11 @@
       <c r="C82" s="2">
         <v>8</v>
       </c>
-      <c r="D82" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D82" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>82</v>
       </c>
@@ -2223,12 +2033,11 @@
       <c r="C83" s="2">
         <v>8</v>
       </c>
-      <c r="D83" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D83" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>83</v>
       </c>
@@ -2238,12 +2047,11 @@
       <c r="C84" s="2">
         <v>8</v>
       </c>
-      <c r="D84" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D84" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>84</v>
       </c>
@@ -2253,12 +2061,11 @@
       <c r="C85" s="2">
         <v>8</v>
       </c>
-      <c r="D85" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D85" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>85</v>
       </c>
@@ -2268,12 +2075,11 @@
       <c r="C86" s="2">
         <v>8</v>
       </c>
-      <c r="D86" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D86" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>86</v>
       </c>
@@ -2283,12 +2089,11 @@
       <c r="C87" s="2">
         <v>8</v>
       </c>
-      <c r="D87" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D87" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>87</v>
       </c>
@@ -2298,23 +2103,11 @@
       <c r="C88" s="2">
         <v>8</v>
       </c>
-      <c r="D88" s="2" t="str">
-        <f t="shared" ref="D88:D93" si="2">IF(C51="Pilates",1,
-IF(C51="Yoga",2,
-IF(C51="Fitness &amp; Musculation",3,
-IF(C51="Escalade",5,
-IF(C51="Boxe",6,
-IF(C51="Danse",7,
-IF(C51="Gymnastique",8,
-IF(C51="Activité Physique Adaptée (APA)",9,
-IF(C51="Bien-Être &amp; Récupération",10,
-IF(C51="Activités aquatiques",11,
-IF(C51="Animation &amp; Encadrement sportif",4,""))))))))))
-)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D88" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>88</v>
       </c>
@@ -2324,12 +2117,11 @@
       <c r="C89" s="2">
         <v>8</v>
       </c>
-      <c r="D89" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D89" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>89</v>
       </c>
@@ -2339,12 +2131,11 @@
       <c r="C90" s="2">
         <v>8</v>
       </c>
-      <c r="D90" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D90" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>90</v>
       </c>
@@ -2354,12 +2145,11 @@
       <c r="C91" s="2">
         <v>8</v>
       </c>
-      <c r="D91" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D91" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>91</v>
       </c>
@@ -2369,12 +2159,11 @@
       <c r="C92" s="2">
         <v>8</v>
       </c>
-      <c r="D92" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="D92" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>92</v>
       </c>
@@ -2384,12 +2173,12 @@
       <c r="C93" s="2">
         <v>8</v>
       </c>
-      <c r="D93" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="D93" s="5" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>